<commit_message>
incorporación de diccionario a etapa 1, creación planilla cierre de ot
</commit_message>
<xml_diff>
--- a/output/_temp/etapa_1_limpieza_base/Cierre de OT Turno 19.03 al 25.03.xlsx
+++ b/output/_temp/etapa_1_limpieza_base/Cierre de OT Turno 19.03 al 25.03.xlsx
@@ -7505,7 +7505,11 @@
         <v/>
       </c>
       <c r="K38" s="4" t="n"/>
-      <c r="L38" s="4" t="inlineStr"/>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>NF</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -7548,7 +7552,11 @@
         <v/>
       </c>
       <c r="K39" s="4" t="n"/>
-      <c r="L39" s="4" t="inlineStr"/>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>NF</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">

</xml_diff>